<commit_message>
Update Word and workflow files
</commit_message>
<xml_diff>
--- a/Workflows/Chemical validation/Level0_Templates/XXXX_XX_AMMONIUM.xlsx
+++ b/Workflows/Chemical validation/Level0_Templates/XXXX_XX_AMMONIUM.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jtorrens\ICP\repoGitLab\lifewatch-vre\Workflows\Chemical validation\Level0_Templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F5968706-1F15-4A42-8778-159FE23A7D9C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3B627B9A-E56E-483D-993E-C09386E1FD90}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{3FD923B0-A352-4B39-804E-C5D1C21F4722}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{3FD923B0-A352-4B39-804E-C5D1C21F4722}"/>
   </bookViews>
   <sheets>
     <sheet name="Readme" sheetId="2" r:id="rId1"/>
@@ -554,7 +554,7 @@
               <a:ea typeface="+mn-ea"/>
               <a:cs typeface="+mn-cs"/>
             </a:rPr>
-            <a:t>Use the standardised ICP sample code for the plot and subprogramme. The code combines the plot number, the species abbreviation, the collection type (INT = interior/throughfall, EXT = exterior/bulk deposition) and any additional qualifier: INT         = throughfall (interior of the forest) EXT         = bulk open-field deposition (exterior) NIEVE       = snow sample LIX 20      = soil lysimeter at 20 cm depth LIX 60      = soil lysimeter at 60 cm depth LIX G 20    = gravity lysimeter at 20 cm depth LIX G 60    = gravity lysimeter at 60 cm depth</a:t>
+            <a:t>Use the standardised ICP sample code for the plot and subprogramme. The code could combines the plot number, the species abbreviation, the collection type (INT = interior/throughfall, EXT = exterior/bulk deposition) and any additional qualifier: INT         = throughfall (interior of the forest) EXT         = bulk open-field deposition (exterior) NIEVE       = snow sample LIX 20      = soil lysimeter at 20 cm depth LIX 60      = soil lysimeter at 60 cm depth LIX G 20    = gravity lysimeter at 20 cm depth LIX G 60    = gravity lysimeter at 60 cm depth</a:t>
           </a:r>
           <a:endParaRPr lang="es-ES" sz="1100">
             <a:solidFill>
@@ -711,6 +711,18 @@
             <a:t>- How to fill: </a:t>
           </a:r>
           <a:r>
+            <a:rPr lang="en-US" sz="1100" b="0">
+              <a:solidFill>
+                <a:schemeClr val="dk1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>You could u</a:t>
+          </a:r>
+          <a:r>
             <a:rPr lang="en-US" sz="1100">
               <a:solidFill>
                 <a:schemeClr val="dk1"/>
@@ -720,7 +732,7 @@
               <a:ea typeface="+mn-ea"/>
               <a:cs typeface="+mn-cs"/>
             </a:rPr>
-            <a:t>Use the official ICP plot number (e.g. 05, 22, 115). Do not include leading zeros beyond the standard format.</a:t>
+            <a:t>se the official ICP plot number (e.g. 05, 22, 115).</a:t>
           </a:r>
           <a:endParaRPr lang="es-ES" sz="1100">
             <a:solidFill>
@@ -1628,7 +1640,31 @@
               <a:ea typeface="+mn-ea"/>
               <a:cs typeface="+mn-cs"/>
             </a:rPr>
-            <a:t>Ammonium-nitrogen concentration measured by the laboratory, expressed in mg/L as N (nitrogen basis, not as NH4+).</a:t>
+            <a:t>Ammonium-nitrogen concentration measured by the laboratory, expressed in </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="1">
+              <a:solidFill>
+                <a:schemeClr val="dk1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>mg/L </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="dk1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>as N (nitrogen basis, not as NH4+).</a:t>
           </a:r>
           <a:endParaRPr lang="es-ES" sz="1100">
             <a:solidFill>
@@ -1663,7 +1699,7 @@
               <a:ea typeface="+mn-ea"/>
               <a:cs typeface="+mn-cs"/>
             </a:rPr>
-            <a:t>Enter the numeric value reported by the laboratory. Use a decimal point (not a comma) as the decimal separator. If the value is below the detection limit, enter the value as reported — the LOQ substitution is applied automatically by the workflow. If the measurement was not performed or the sample was lost, leave the cell empty (do not enter 0 or n.a.).</a:t>
+            <a:t>Enter the numeric value reported by the laboratory. If the value is below the detection limit, enter the value as reported — the LOQ substitution is applied automatically by the workflow. If the measurement was not performed or the sample was lost, leave the cell empty (do not enter 0 or n.a.).</a:t>
           </a:r>
           <a:endParaRPr lang="es-ES" sz="1100">
             <a:solidFill>

</xml_diff>